<commit_message>
Shortened functions, TB paths now copy SV
</commit_message>
<xml_diff>
--- a/excel_utils/outputs/worklist_conditions_project_12.xlsx
+++ b/excel_utils/outputs/worklist_conditions_project_12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/excel_utils/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E6D56C-7335-CD48-80B4-1FAF357C8229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6113EE9-8A04-974C-B723-860ACF006BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3100" yWindow="680" windowWidth="24040" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3100" yWindow="680" windowWidth="24040" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -291,7 +291,7 @@
     <t>C:\Xcalibur\methods\XiaoFeng\2029</t>
   </si>
   <si>
-    <t>5-9</t>
+    <t>5-10</t>
   </si>
 </sst>
 </file>

</xml_diff>